<commit_message>
Added automatic matura upload
</commit_message>
<xml_diff>
--- a/OnlineExamer.Web/wwwroot/Maturi/xlsx/Български език_2014.xlsx
+++ b/OnlineExamer.Web/wwwroot/Maturi/xlsx/Български език_2014.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Матури\xlsx\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Examer\OnlineExamer.Web\wwwroot\Maturi\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{117468DC-8B53-4A1C-BF98-8EB92D8800CA}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DB843DC-1040-4261-8EE4-0D5D5EFA5188}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{2F88FA51-3A67-4843-81CC-93A859985177}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
   <si>
     <t>1. В кой от редовете е допусната правописна грешка?</t>
   </si>
@@ -108,9 +108,6 @@
   </si>
   <si>
     <t>Г) Един от основните белези на Просвещението е неговата свързаност с науката.</t>
-  </si>
-  <si>
-    <t>6. В коя от подчертаните думи е допусната граматична грешка?  Няколко работници (А) от фирмата за почистване на пътищата се бяха събрали около  четирите автомобила (Б), закъсали в снега. До тях двама полицая (В) спираха  движението, за да работят нормално двата снегорина (Г).</t>
   </si>
   <si>
     <t>А)</t>
@@ -535,10 +532,40 @@
     <t>В) Необходимо е хлябът и всички видове макаронени и тестени изделия да бъдат  изключени от менюто в ученическите столове.</t>
   </si>
   <si>
-    <t>Г) На учениците е необходимо да се осигури консумация на пълнозърнести макаронени  продукти най-малко веднъж седмично.    3</t>
-  </si>
-  <si>
     <t>Г) сравнение</t>
+  </si>
+  <si>
+    <t>Въпрос</t>
+  </si>
+  <si>
+    <t>Отговор А</t>
+  </si>
+  <si>
+    <t>Отговор Б</t>
+  </si>
+  <si>
+    <t>Отговор В</t>
+  </si>
+  <si>
+    <t>Отговор Г</t>
+  </si>
+  <si>
+    <t>Отговор</t>
+  </si>
+  <si>
+    <t>Точки</t>
+  </si>
+  <si>
+    <t>Единичен отговор</t>
+  </si>
+  <si>
+    <t>Отворен отговор</t>
+  </si>
+  <si>
+    <t>Г) На учениците е необходимо да се осигури консумация на пълнозърнести макаронени  продукти най-малко веднъж седмично.</t>
+  </si>
+  <si>
+    <t>6. В коя от подчертаните думи е допусната граматична грешка?  Няколко РАБОТНИЦИ (А) от фирмата за почистване на пътищата се бяха събрали около  четирите АВТОМОБИЛА (Б), закъсали в снега. До тях двама ПОЛИЦАЯ (В) спираха  движението, за да работят нормално двата СНЕГОРИНА (Г).</t>
   </si>
 </sst>
 </file>
@@ -575,10 +602,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -894,7 +924,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C5FA935-ED1B-4EC5-AEDC-DC9D9B328084}">
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="255.77734375" bestFit="1" customWidth="1"/>
@@ -902,613 +932,918 @@
     <col min="3" max="3" width="114" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="116.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="118.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="F1">
+      <c r="F2">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E3" t="s">
         <v>9</v>
       </c>
-      <c r="F2">
+      <c r="F3">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E4" t="s">
         <v>14</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D5" t="s">
         <v>18</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E5" t="s">
         <v>19</v>
       </c>
-      <c r="F4">
+      <c r="F5">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>22</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>23</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E6" t="s">
         <v>24</v>
       </c>
-      <c r="F5">
+      <c r="F6">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>160</v>
+      </c>
+      <c r="B7" t="s">
         <v>25</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D7" t="s">
         <v>27</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E7" t="s">
         <v>28</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F7">
+        <v>3</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>29</v>
       </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="B8" t="s">
         <v>30</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C8" t="s">
         <v>31</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D8" t="s">
         <v>32</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E8" t="s">
         <v>33</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>34</v>
       </c>
-      <c r="F7">
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" t="s">
+        <v>47</v>
+      </c>
+      <c r="E11" t="s">
+        <v>48</v>
+      </c>
+      <c r="F11">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" t="s">
-        <v>39</v>
-      </c>
-      <c r="F8">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" t="s">
-        <v>43</v>
-      </c>
-      <c r="E9" t="s">
-        <v>44</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" t="s">
-        <v>46</v>
-      </c>
-      <c r="C10" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" t="s">
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>49</v>
       </c>
-      <c r="F10">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="B12" t="s">
         <v>50</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C12" t="s">
         <v>51</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D12" t="s">
         <v>52</v>
       </c>
-      <c r="D11" t="s">
+      <c r="E12" t="s">
         <v>53</v>
-      </c>
-      <c r="E11" t="s">
-        <v>54</v>
-      </c>
-      <c r="F11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B12" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" t="s">
-        <v>59</v>
       </c>
       <c r="F12">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" t="s">
+        <v>58</v>
+      </c>
+      <c r="F13">
+        <v>3</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>1</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" t="s">
         <v>60</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C14" t="s">
         <v>61</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D14" t="s">
         <v>62</v>
       </c>
-      <c r="D13" t="s">
+      <c r="E14" t="s">
         <v>63</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>64</v>
       </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="B15" t="s">
         <v>65</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C15" t="s">
         <v>66</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D15" t="s">
         <v>67</v>
       </c>
-      <c r="D14" t="s">
+      <c r="E15" t="s">
         <v>68</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>69</v>
       </c>
-      <c r="F14">
+      <c r="B16" t="s">
+        <v>70</v>
+      </c>
+      <c r="C16" t="s">
+        <v>71</v>
+      </c>
+      <c r="D16" t="s">
+        <v>72</v>
+      </c>
+      <c r="E16" t="s">
+        <v>73</v>
+      </c>
+      <c r="F16">
+        <v>4</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" t="s">
+        <v>76</v>
+      </c>
+      <c r="D17" t="s">
+        <v>77</v>
+      </c>
+      <c r="E17" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17">
         <v>3</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D15" t="s">
-        <v>73</v>
-      </c>
-      <c r="E15" t="s">
-        <v>74</v>
-      </c>
-      <c r="F15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
-        <v>75</v>
-      </c>
-      <c r="B16" t="s">
-        <v>76</v>
-      </c>
-      <c r="C16" t="s">
-        <v>77</v>
-      </c>
-      <c r="D16" t="s">
-        <v>78</v>
-      </c>
-      <c r="E16" t="s">
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>1</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>79</v>
       </c>
-      <c r="F16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="B18" t="s">
         <v>80</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C18" t="s">
         <v>81</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D18" t="s">
         <v>82</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E18" t="s">
         <v>83</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>84</v>
       </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="B19" t="s">
         <v>85</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C19" t="s">
         <v>86</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D19" t="s">
         <v>87</v>
       </c>
-      <c r="D18" t="s">
+      <c r="E19" t="s">
         <v>88</v>
-      </c>
-      <c r="E18" t="s">
-        <v>89</v>
-      </c>
-      <c r="F18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" t="s">
-        <v>91</v>
-      </c>
-      <c r="C19" t="s">
-        <v>92</v>
-      </c>
-      <c r="D19" t="s">
-        <v>93</v>
-      </c>
-      <c r="E19" t="s">
-        <v>94</v>
       </c>
       <c r="F19">
         <v>4</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>89</v>
+      </c>
+      <c r="B20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" t="s">
+        <v>91</v>
+      </c>
+      <c r="D20" t="s">
+        <v>92</v>
+      </c>
+      <c r="E20" t="s">
+        <v>93</v>
+      </c>
+      <c r="F20">
+        <v>4</v>
+      </c>
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>1</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" t="s">
         <v>95</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C21" t="s">
         <v>96</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D21" t="s">
         <v>97</v>
       </c>
-      <c r="D20" t="s">
+      <c r="E21" t="s">
         <v>98</v>
-      </c>
-      <c r="E20" t="s">
-        <v>99</v>
-      </c>
-      <c r="F20">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>100</v>
-      </c>
-      <c r="B21" t="s">
-        <v>101</v>
-      </c>
-      <c r="C21" t="s">
-        <v>102</v>
-      </c>
-      <c r="D21" t="s">
-        <v>103</v>
-      </c>
-      <c r="E21" t="s">
-        <v>104</v>
       </c>
       <c r="F21">
         <v>3</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>1</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" t="s">
+        <v>102</v>
+      </c>
+      <c r="E22" t="s">
+        <v>103</v>
+      </c>
+      <c r="F22">
+        <v>3</v>
+      </c>
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>1</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>104</v>
+      </c>
+      <c r="B23" t="s">
         <v>105</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C23" t="s">
         <v>106</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D23" t="s">
         <v>107</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E23" t="s">
+        <v>149</v>
+      </c>
+      <c r="F23">
+        <v>2</v>
+      </c>
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>1</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="403.2" x14ac:dyDescent="0.3">
+      <c r="A24" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E22" t="s">
-        <v>151</v>
-      </c>
-      <c r="F22">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="403.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="1" t="s">
+    </row>
+    <row r="25" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="A25" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="345.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="1" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="B26" t="s">
         <v>111</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C26" t="s">
         <v>112</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D26" t="s">
         <v>113</v>
       </c>
-      <c r="D25" t="s">
+      <c r="E26" t="s">
         <v>114</v>
-      </c>
-      <c r="E25" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>116</v>
-      </c>
-      <c r="B26" t="s">
-        <v>117</v>
-      </c>
-      <c r="C26" t="s">
-        <v>118</v>
-      </c>
-      <c r="D26" t="s">
-        <v>119</v>
-      </c>
-      <c r="E26" t="s">
-        <v>120</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>1</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="B27" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C27" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="D27" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="E27" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="F27">
         <v>3</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G27">
+        <v>1</v>
+      </c>
+      <c r="H27">
+        <v>1</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" t="s">
+        <v>121</v>
+      </c>
+      <c r="C28" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" t="s">
+        <v>124</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28">
+        <v>1</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" t="s">
         <v>126</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C29" t="s">
         <v>127</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D29" t="s">
         <v>128</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E29" t="s">
         <v>129</v>
       </c>
-      <c r="E28" t="s">
+      <c r="F29">
+        <v>3</v>
+      </c>
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>1</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
         <v>130</v>
       </c>
-      <c r="F28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
+      <c r="B30" t="s">
         <v>131</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C30" t="s">
         <v>132</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D30" t="s">
         <v>133</v>
       </c>
-      <c r="D29" t="s">
+      <c r="E30" t="s">
         <v>134</v>
       </c>
-      <c r="E29" t="s">
+      <c r="F30">
+        <v>4</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>1</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
         <v>135</v>
       </c>
-      <c r="F29">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
+      <c r="B31" t="s">
         <v>136</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C31" t="s">
         <v>137</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D31" t="s">
         <v>138</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E31" t="s">
         <v>139</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>1</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>140</v>
       </c>
-      <c r="F30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
+      <c r="B32" t="s">
         <v>141</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C32" t="s">
         <v>142</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D32" t="s">
         <v>143</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E32" t="s">
         <v>144</v>
       </c>
-      <c r="E31" t="s">
+      <c r="F32">
+        <v>2</v>
+      </c>
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32">
+        <v>1</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
         <v>145</v>
       </c>
-      <c r="F31">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
+      <c r="B33" t="s">
         <v>146</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C33" t="s">
         <v>147</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D33" t="s">
         <v>148</v>
       </c>
-      <c r="D32" t="s">
-        <v>149</v>
-      </c>
-      <c r="E32" t="s">
-        <v>150</v>
-      </c>
-      <c r="F32">
+      <c r="E33" t="s">
+        <v>159</v>
+      </c>
+      <c r="F33">
         <v>3</v>
+      </c>
+      <c r="G33">
+        <v>1</v>
+      </c>
+      <c r="H33">
+        <v>1</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>